<commit_message>
Daily EOD data and reports for 2026-09-03
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260903.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260903.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.915</v>
+        <v>1.92</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.02</v>
+        <v>0.025</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1.06%</t>
+          <t>1.32%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>293341.61</v>
+        <v>294107.52</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>3063.62</v>
+        <v>3829.52</v>
       </c>
     </row>
     <row r="5">
@@ -569,24 +569,24 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>63.8</v>
+        <v>63.78</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>-0.85</v>
+        <v>-0.87</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>-1.31%</t>
+          <t>-1.35%</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
         <v>9000</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>574200</v>
+        <v>574020</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>-7650</v>
+        <v>-7830</v>
       </c>
     </row>
     <row r="8">
@@ -623,14 +623,14 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>161.06</v>
+        <v>160.58</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>1.74</v>
+        <v>1.26</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.09%</t>
+          <t>0.79%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -650,24 +650,24 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>0.975</v>
+        <v>0.985</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.015</v>
+        <v>0.025</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.56%</t>
+          <t>2.60%</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
         <v>10000</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>9750</v>
+        <v>9850</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>150</v>
+        <v>250</v>
       </c>
     </row>
     <row r="11">
@@ -677,24 +677,24 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>174.94</v>
+        <v>175.5</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>1.09</v>
+        <v>1.65</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.63%</t>
+          <t>0.95%</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>699760</v>
+        <v>702000</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>4360</v>
+        <v>6600</v>
       </c>
     </row>
     <row r="12">
@@ -758,24 +758,24 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>0.117</v>
+        <v>0.12</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>-0.003</v>
+        <v>0</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>-2.50%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E14" s="3" t="n">
         <v>9412</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>1101.2</v>
+        <v>1129.44</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>-28.24</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -785,24 +785,24 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>0.1</v>
+        <v>0.095</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.001</v>
+        <v>-0.004</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>1.01%</t>
+          <t>-4.04%</t>
         </is>
       </c>
       <c r="E15" s="3" t="n">
         <v>6000</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>600</v>
+        <v>570</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>6</v>
+        <v>-24</v>
       </c>
     </row>
     <row r="16">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>35.015</v>
+        <v>34.91</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.625</v>
+        <v>0.52</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1.82%</t>
+          <t>1.51%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>32.01</v>
+        <v>32.22</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>-1.07</v>
+        <v>-0.86</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>-3.23%</t>
+          <t>-2.60%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>41228.88</v>
+        <v>41499.36</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>-1378.16</v>
+        <v>-1107.68</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1795702.15</v>
+        <v>1798896.77</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>-72758.55</v>
+        <v>-69563.92999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Reduce BHP holding to 8000 units from 2026-09-03
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260903.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260903.xlsx
@@ -580,13 +580,13 @@
         </is>
       </c>
       <c r="E7" s="3" t="n">
-        <v>9000</v>
+        <v>8000</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>574020</v>
+        <v>510240</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>-7830</v>
+        <v>-6960</v>
       </c>
     </row>
     <row r="8">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1867522.63</v>
+        <v>1803742.63</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>-938.0700000000001</v>
+        <v>-68.06999999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>